<commit_message>
docs(wallet): sync data dictionary to 20 tables (auth + wallet + vault)
</commit_message>
<xml_diff>
--- a/.claude/docs/vaultpay-data-dictionary.xlsx
+++ b/.claude/docs/vaultpay-data-dictionary.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="auth-columns" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wallet-columns" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vault-columns" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -992,6 +993,60 @@
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>From/to wallets, amount, currency, status (PENDING/COMPLETED/FAILED/REVERSED) and a unique reference; links the two transaction legs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>vault</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Metadata for an uploaded document.</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>The encrypted file lives in MinIO; the service needs a queryable record of ownership, name, size, checksum and status.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Per-document row: user_id (plain ref), original filename, MinIO storage_key, mime type, plaintext size, sha256 checksum, category and soft-delete status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>vault</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Time-limited public share links for a document.</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Owners can share a document without exposing their JWT; tokens must be revocable, expiring and download-limited.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Hashed share token with optional expiry and max-downloads, a download counter, creator and revocation timestamp.</t>
         </is>
       </c>
     </row>
@@ -5023,4 +5078,626 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>vault-service — column dictionary</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Constraints</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Primary key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>indexed</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Owner — plain reference to auth users.id (no cross-DB FK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>filename</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Original upload filename.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>storage_key</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>UNIQUE, NOT NULL</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Object key in MinIO (holds ciphertext).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>mime_type</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Reported content type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>size_bytes</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Plaintext size in bytes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>checksum</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>sha256 of plaintext; verified on download.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Optional user category/tag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>default ACTIVE</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE | DELETED (soft delete; blob retained).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Upload time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>@updatedAt</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Last update time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Soft-delete marker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Primary key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>document_id</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>FK documents.id</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Shared document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>token_hash</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>UNIQUE, NOT NULL</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>sha256 of the share token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>created_by</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>User who created the share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>expires_at</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Optional expiry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>max_downloads</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Optional download cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>download_count</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>default 0</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Downloads used so far.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>revoked_at</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Set when revoked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>document_shares</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Creation time.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(wallet): sync data dictionary to 21 tables (+admin)
</commit_message>
<xml_diff>
--- a/.claude/docs/vaultpay-data-dictionary.xlsx
+++ b/.claude/docs/vaultpay-data-dictionary.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="auth-columns" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wallet-columns" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vault-columns" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="admin-columns" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1047,6 +1048,33 @@
       <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Hashed share token with optional expiry and max-downloads, a download counter, creator and revocation timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Audit trail of back-office admin actions.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Staff actions (viewing/suspending customers, etc.) must be attributable and reviewable for compliance.</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Append-only rows: which admin did what action to which target, with IP and metadata; customer data itself is fetched from auth over S2S, not stored here.</t>
         </is>
       </c>
     </row>
@@ -5700,4 +5728,302 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>admin-service — column dictionary</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Constraints</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Primary key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>admin_id</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>indexed</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Acting admin (ref to auth admin_users.id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>admin_email</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Admin email at action time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>indexed</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Action code (e.g. CUSTOMER_SUSPENDED).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>target_type</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Target kind (e.g. CUSTOMER).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>target_id</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Target identifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Extra action context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ip</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Admin client IP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>admin_activity_logs</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>default now()</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Action time.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>